<commit_message>
Day 4 delivarable added
</commit_message>
<xml_diff>
--- a/Sprint/src/test/resources/Data/redbus_test_data_sdc.xlsx
+++ b/Sprint/src/test/resources/Data/redbus_test_data_sdc.xlsx
@@ -3,26 +3,21 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Soumy\OneDrive\Desktop\Workspace3\redbus\src\test\resources\testdata\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD245B8D-AD6F-4B82-A568-87252A664796}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{E4787BD1-9D00-4E91-A9EA-CBFF0ECE846C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="18240" windowHeight="7392" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="11400" windowHeight="7392" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BusSearch" sheetId="1" r:id="rId1"/>
     <sheet name="SearchResults" sheetId="2" r:id="rId2"/>
-    <sheet name="Background" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
+  <oleSize ref="A1:G23"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="45">
   <si>
     <t>testCaseId</t>
   </si>
@@ -102,9 +97,6 @@
     <t>SR_01</t>
   </si>
   <si>
-    <t>AC</t>
-  </si>
-  <si>
     <t>SEATER</t>
   </si>
   <si>
@@ -151,9 +143,6 @@
   </si>
   <si>
     <t>Evening</t>
-  </si>
-  <si>
-    <t>dummy</t>
   </si>
   <si>
     <t>SR_07</t>
@@ -614,7 +603,7 @@
         <v>6</v>
       </c>
       <c r="D2" s="7">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E2" s="5"/>
       <c r="F2" s="5"/>
@@ -641,7 +630,7 @@
         <v>11</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D4" s="7"/>
       <c r="E4" s="5"/>
@@ -667,10 +656,10 @@
         <v>6</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D6" s="7">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E6" s="5"/>
       <c r="F6" s="5"/>
@@ -707,7 +696,7 @@
         <v>8</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D9" s="7"/>
       <c r="E9" s="5"/>
@@ -721,7 +710,7 @@
         <v>18</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D10" s="7"/>
       <c r="E10" s="5"/>
@@ -738,7 +727,7 @@
         <v>6</v>
       </c>
       <c r="D11" s="7">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E11" s="5"/>
       <c r="F11" s="5"/>
@@ -748,7 +737,7 @@
         <v>20</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C12" s="7"/>
       <c r="D12" s="7"/>
@@ -798,7 +787,7 @@
         <v>24</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="F1" s="1"/>
     </row>
@@ -807,10 +796,10 @@
         <v>25</v>
       </c>
       <c r="B2" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="C2" s="10" t="s">
         <v>26</v>
-      </c>
-      <c r="C2" s="10" t="s">
-        <v>27</v>
       </c>
       <c r="D2" s="10"/>
       <c r="E2" s="10"/>
@@ -818,13 +807,13 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="C3" s="10" t="s">
         <v>28</v>
-      </c>
-      <c r="B3" s="10" t="s">
-        <v>41</v>
-      </c>
-      <c r="C3" s="10" t="s">
-        <v>29</v>
       </c>
       <c r="D3" s="10"/>
       <c r="E3" s="10"/>
@@ -832,10 +821,10 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="10" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C4" s="10"/>
       <c r="D4" s="10"/>
@@ -844,49 +833,49 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B5" s="10"/>
       <c r="C5" s="10"/>
       <c r="D5" s="10" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E5" s="10"/>
       <c r="F5" s="2"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B6" s="10"/>
       <c r="C6" s="10"/>
       <c r="D6" s="10" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E6" s="10"/>
       <c r="F6" s="2"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="10" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B7" s="10"/>
       <c r="C7" s="10"/>
       <c r="D7" s="10" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E7" s="10"/>
       <c r="F7" s="2"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="10" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B8" s="10"/>
       <c r="C8" s="10"/>
       <c r="D8" s="10"/>
       <c r="E8" s="10" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="F8" s="2"/>
     </row>
@@ -894,37 +883,4 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="2" width="14" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" s="2"/>
-      <c r="B2" s="2"/>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Day 6 delivarable added
</commit_message>
<xml_diff>
--- a/Sprint/src/test/resources/Data/redbus_test_data_sdc.xlsx
+++ b/Sprint/src/test/resources/Data/redbus_test_data_sdc.xlsx
@@ -3,16 +3,16 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{E4787BD1-9D00-4E91-A9EA-CBFF0ECE846C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{2E3D61F0-B79C-4CEE-B0DB-0B6FDF4C8E6D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="11400" windowHeight="7392" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="12660" windowHeight="7392" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BusSearch" sheetId="1" r:id="rId1"/>
     <sheet name="SearchResults" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A1:G23"/>
+  <oleSize ref="A1:H23"/>
 </workbook>
 </file>
 
@@ -603,7 +603,7 @@
         <v>6</v>
       </c>
       <c r="D2" s="7">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E2" s="5"/>
       <c r="F2" s="5"/>
@@ -659,7 +659,7 @@
         <v>36</v>
       </c>
       <c r="D6" s="7">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E6" s="5"/>
       <c r="F6" s="5"/>
@@ -727,7 +727,7 @@
         <v>6</v>
       </c>
       <c r="D11" s="7">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E11" s="5"/>
       <c r="F11" s="5"/>

</xml_diff>